<commit_message>
Mise à jour profils suite erreurs QA IPS a14d09011e46756bf6f25a40d45539aa00ff470c
</commit_message>
<xml_diff>
--- a/correctionProfile/ig/StructureDefinition-fr-observation-assessment-document.xlsx
+++ b/correctionProfile/ig/StructureDefinition-fr-observation-assessment-document.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$110</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5463" uniqueCount="673">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4208" uniqueCount="615">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-29T08:08:01+00:00</t>
+    <t>2026-09-29T09:01:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1807,11 +1807,11 @@
     <t>Observation.hasMember</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Observation|4.0.1|QuestionnaireResponse|4.0.1|MolecularSequence|4.0.1)
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-observation-assessment-document|0.1.0)
 </t>
   </si>
   <si>
-    <t>Référence interne</t>
+    <t>Sous-évaluations (composants N2) rattachées à cette évaluation N1</t>
   </si>
   <si>
     <t>This observation is a group observation (e.g. a battery, a panel of tests, a set of vital sign measurements) that includes the target as a member of the group.</t>
@@ -1848,7 +1848,7 @@
     <t>Observation.component</t>
   </si>
   <si>
-    <t>Composants de l'évaluation</t>
+    <t>Component results</t>
   </si>
   <si>
     <t>Some observations have multiple component observations.  These component observations are expressed as separate code value pairs that share the same attributes.  Examples include systolic and diastolic component observations for blood pressure measurement and multiple component observations for genetics observations.</t>
@@ -1858,10 +1858,6 @@
   </si>
   <si>
     <t>Component observations share the same attributes in the Observation resource as the primary observation and are always treated a part of a single observation (they are not separable).   However, the reference range for the primary observation value is not inherited by the component values and is required when appropriate for each component observation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pattern:extension('https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-evaluation-level-extension').value}
-</t>
   </si>
   <si>
     <t>containment by OBX-4?</t>
@@ -1939,179 +1935,6 @@
   </si>
   <si>
     <t>Guidance on how to interpret the value by comparison to a normal or recommended range.</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1</t>
-  </si>
-  <si>
-    <t>ComposantN1</t>
-  </si>
-  <si>
-    <t>Composant N1 de l'évaluation</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.id</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:evaluationLevel</t>
-  </si>
-  <si>
-    <t>evaluationLevel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-evaluation-level-extension|0.1.0}
-</t>
-  </si>
-  <si>
-    <t>FR Evaluation Level Extension</t>
-  </si>
-  <si>
-    <t>Extension permettant d'indiquer le niveau (N1 ou N2) d'un composant d'une évaluation.</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:evaluationLevel.id</t>
-  </si>
-  <si>
-    <t>Observation.component.extension.id</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:evaluationLevel.extension</t>
-  </si>
-  <si>
-    <t>Observation.component.extension.extension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:evaluationLevel.url</t>
-  </si>
-  <si>
-    <t>Observation.component.extension.url</t>
-  </si>
-  <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/document-core/StructureDefinition/fr-evaluation-level-extension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:evaluationLevel.value[x]</t>
-  </si>
-  <si>
-    <t>Observation.component.extension.value[x]</t>
-  </si>
-  <si>
-    <t>N1</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:note</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {note|5.3.0}
-</t>
-  </si>
-  <si>
-    <t>Commentaire</t>
-  </si>
-  <si>
-    <t>Additional notes that apply to this resource or element.</t>
-  </si>
-  <si>
-    <t>This extension SHALL NOT be used if the resource already has standard 'note' element (or equivalent) of type Annotation on the same element</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:note.id</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:note.extension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:note.url</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/StructureDefinition/note</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.extension:note.value[x]</t>
-  </si>
-  <si>
-    <t>Notes for this resource/element</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.modifierExtension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.code</t>
-  </si>
-  <si>
-    <t>Code de l'évaluation</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.value[x]</t>
-  </si>
-  <si>
-    <t>Résultat de l'évaluation</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.dataAbsentReason</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.interpretation</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN1.referenceRange</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2</t>
-  </si>
-  <si>
-    <t>ComposantN2</t>
-  </si>
-  <si>
-    <t>Sous-composant N2 de l'évaluation</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.id</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.extension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.extension:evaluationLevel</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.extension:evaluationLevel.id</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.extension:evaluationLevel.extension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.extension:evaluationLevel.url</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.extension:evaluationLevel.value[x]</t>
-  </si>
-  <si>
-    <t>N2</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.modifierExtension</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.code</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.value[x]</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.dataAbsentReason</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.interpretation</t>
-  </si>
-  <si>
-    <t>Observation.component:ComposantN2.referenceRange</t>
   </si>
 </sst>
 </file>
@@ -2428,12 +2251,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP143"/>
+  <dimension ref="A1:AP110"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="67.41796875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="50.2890625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="13.33984375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="11.5234375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -2458,7 +2281,7 @@
     <col min="25" max="25" width="54.6171875" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="74.97265625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="102.171875" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="36.0390625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>
@@ -14583,7 +14406,7 @@
         <v>81</v>
       </c>
       <c r="H102" t="s" s="2">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="I102" t="s" s="2">
         <v>82</v>
@@ -14641,14 +14464,16 @@
         <v>82</v>
       </c>
       <c r="AB102" t="s" s="2">
-        <v>590</v>
-      </c>
-      <c r="AC102" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="AC102" t="s" s="2">
+        <v>82</v>
+      </c>
       <c r="AD102" t="s" s="2">
         <v>82</v>
       </c>
       <c r="AE102" t="s" s="2">
-        <v>142</v>
+        <v>82</v>
       </c>
       <c r="AF102" t="s" s="2">
         <v>585</v>
@@ -14672,10 +14497,10 @@
         <v>82</v>
       </c>
       <c r="AM102" t="s" s="2">
+        <v>590</v>
+      </c>
+      <c r="AN102" t="s" s="2">
         <v>591</v>
-      </c>
-      <c r="AN102" t="s" s="2">
-        <v>592</v>
       </c>
       <c r="AO102" t="s" s="2">
         <v>82</v>
@@ -14686,10 +14511,10 @@
     </row>
     <row r="103" hidden="true">
       <c r="A103" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B103" t="s" s="2">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" t="s" s="2">
@@ -14804,10 +14629,10 @@
     </row>
     <row r="104" hidden="true">
       <c r="A104" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B104" t="s" s="2">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C104" s="2"/>
       <c r="D104" t="s" s="2">
@@ -14924,10 +14749,10 @@
     </row>
     <row r="105" hidden="true">
       <c r="A105" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B105" t="s" s="2">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C105" s="2"/>
       <c r="D105" t="s" s="2">
@@ -15046,10 +14871,10 @@
     </row>
     <row r="106" hidden="true">
       <c r="A106" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B106" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" t="s" s="2">
@@ -15075,13 +14900,13 @@
         <v>190</v>
       </c>
       <c r="L106" t="s" s="2">
+        <v>596</v>
+      </c>
+      <c r="M106" t="s" s="2">
         <v>597</v>
       </c>
-      <c r="M106" t="s" s="2">
+      <c r="N106" t="s" s="2">
         <v>598</v>
-      </c>
-      <c r="N106" t="s" s="2">
-        <v>599</v>
       </c>
       <c r="O106" t="s" s="2">
         <v>377</v>
@@ -15112,11 +14937,11 @@
         <v>485</v>
       </c>
       <c r="Y106" t="s" s="2">
+        <v>599</v>
+      </c>
+      <c r="Z106" t="s" s="2">
         <v>600</v>
       </c>
-      <c r="Z106" t="s" s="2">
-        <v>601</v>
-      </c>
       <c r="AA106" t="s" s="2">
         <v>82</v>
       </c>
@@ -15133,7 +14958,7 @@
         <v>82</v>
       </c>
       <c r="AF106" t="s" s="2">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="AG106" t="s" s="2">
         <v>93</v>
@@ -15151,7 +14976,7 @@
         <v>82</v>
       </c>
       <c r="AL106" t="s" s="2">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AM106" t="s" s="2">
         <v>382</v>
@@ -15168,10 +14993,10 @@
     </row>
     <row r="107" hidden="true">
       <c r="A107" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B107" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" t="s" s="2">
@@ -15197,13 +15022,13 @@
         <v>442</v>
       </c>
       <c r="L107" t="s" s="2">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="M107" t="s" s="2">
         <v>444</v>
       </c>
       <c r="N107" t="s" s="2">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="O107" t="s" s="2">
         <v>446</v>
@@ -15255,7 +15080,7 @@
         <v>82</v>
       </c>
       <c r="AF107" t="s" s="2">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AG107" t="s" s="2">
         <v>80</v>
@@ -15273,7 +15098,7 @@
         <v>82</v>
       </c>
       <c r="AL107" t="s" s="2">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="AM107" t="s" s="2">
         <v>449</v>
@@ -15290,10 +15115,10 @@
     </row>
     <row r="108" hidden="true">
       <c r="A108" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B108" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" t="s" s="2">
@@ -15319,13 +15144,13 @@
         <v>190</v>
       </c>
       <c r="L108" t="s" s="2">
+        <v>607</v>
+      </c>
+      <c r="M108" t="s" s="2">
         <v>608</v>
       </c>
-      <c r="M108" t="s" s="2">
+      <c r="N108" t="s" s="2">
         <v>609</v>
-      </c>
-      <c r="N108" t="s" s="2">
-        <v>610</v>
       </c>
       <c r="O108" t="s" s="2">
         <v>456</v>
@@ -15377,7 +15202,7 @@
         <v>82</v>
       </c>
       <c r="AF108" t="s" s="2">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="AG108" t="s" s="2">
         <v>80</v>
@@ -15412,10 +15237,10 @@
     </row>
     <row r="109" hidden="true">
       <c r="A109" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B109" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="C109" s="2"/>
       <c r="D109" t="s" s="2">
@@ -15441,7 +15266,7 @@
         <v>190</v>
       </c>
       <c r="L109" t="s" s="2">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="M109" t="s" s="2">
         <v>464</v>
@@ -15499,7 +15324,7 @@
         <v>82</v>
       </c>
       <c r="AF109" t="s" s="2">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="AG109" t="s" s="2">
         <v>80</v>
@@ -15534,10 +15359,10 @@
     </row>
     <row r="110" hidden="true">
       <c r="A110" t="s" s="2">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B110" t="s" s="2">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="C110" s="2"/>
       <c r="D110" t="s" s="2">
@@ -15563,10 +15388,10 @@
         <v>83</v>
       </c>
       <c r="L110" t="s" s="2">
+        <v>613</v>
+      </c>
+      <c r="M110" t="s" s="2">
         <v>614</v>
-      </c>
-      <c r="M110" t="s" s="2">
-        <v>615</v>
       </c>
       <c r="N110" t="s" s="2">
         <v>523</v>
@@ -15621,7 +15446,7 @@
         <v>82</v>
       </c>
       <c r="AF110" t="s" s="2">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AG110" t="s" s="2">
         <v>80</v>
@@ -15654,3972 +15479,8 @@
         <v>82</v>
       </c>
     </row>
-    <row r="111" hidden="true">
-      <c r="A111" t="s" s="2">
-        <v>616</v>
-      </c>
-      <c r="B111" t="s" s="2">
-        <v>585</v>
-      </c>
-      <c r="C111" t="s" s="2">
-        <v>617</v>
-      </c>
-      <c r="D111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E111" s="2"/>
-      <c r="F111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G111" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J111" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K111" t="s" s="2">
-        <v>520</v>
-      </c>
-      <c r="L111" t="s" s="2">
-        <v>618</v>
-      </c>
-      <c r="M111" t="s" s="2">
-        <v>587</v>
-      </c>
-      <c r="N111" t="s" s="2">
-        <v>588</v>
-      </c>
-      <c r="O111" t="s" s="2">
-        <v>589</v>
-      </c>
-      <c r="P111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q111" s="2"/>
-      <c r="R111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF111" t="s" s="2">
-        <v>585</v>
-      </c>
-      <c r="AG111" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH111" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ111" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM111" t="s" s="2">
-        <v>591</v>
-      </c>
-      <c r="AN111" t="s" s="2">
-        <v>592</v>
-      </c>
-      <c r="AO111" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP111" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="112" hidden="true">
-      <c r="A112" t="s" s="2">
-        <v>619</v>
-      </c>
-      <c r="B112" t="s" s="2">
-        <v>593</v>
-      </c>
-      <c r="C112" s="2"/>
-      <c r="D112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E112" s="2"/>
-      <c r="F112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G112" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K112" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="L112" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="M112" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="N112" s="2"/>
-      <c r="O112" s="2"/>
-      <c r="P112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q112" s="2"/>
-      <c r="R112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF112" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="AG112" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH112" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN112" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="AO112" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP112" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="113" hidden="true">
-      <c r="A113" t="s" s="2">
-        <v>620</v>
-      </c>
-      <c r="B113" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="C113" s="2"/>
-      <c r="D113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E113" s="2"/>
-      <c r="F113" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G113" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K113" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L113" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="M113" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="N113" s="2"/>
-      <c r="O113" s="2"/>
-      <c r="P113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q113" s="2"/>
-      <c r="R113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB113" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="AC113" s="2"/>
-      <c r="AD113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE113" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AF113" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG113" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH113" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ113" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO113" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP113" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="114" hidden="true">
-      <c r="A114" t="s" s="2">
-        <v>621</v>
-      </c>
-      <c r="B114" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="C114" t="s" s="2">
-        <v>622</v>
-      </c>
-      <c r="D114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E114" s="2"/>
-      <c r="F114" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G114" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K114" t="s" s="2">
-        <v>623</v>
-      </c>
-      <c r="L114" t="s" s="2">
-        <v>624</v>
-      </c>
-      <c r="M114" t="s" s="2">
-        <v>625</v>
-      </c>
-      <c r="N114" s="2"/>
-      <c r="O114" s="2"/>
-      <c r="P114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q114" s="2"/>
-      <c r="R114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF114" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG114" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH114" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI114" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="AJ114" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO114" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP114" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="115" hidden="true">
-      <c r="A115" t="s" s="2">
-        <v>626</v>
-      </c>
-      <c r="B115" t="s" s="2">
-        <v>627</v>
-      </c>
-      <c r="C115" s="2"/>
-      <c r="D115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E115" s="2"/>
-      <c r="F115" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G115" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K115" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="L115" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="M115" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="N115" s="2"/>
-      <c r="O115" s="2"/>
-      <c r="P115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q115" s="2"/>
-      <c r="R115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF115" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="AG115" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH115" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN115" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="AO115" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP115" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="116" hidden="true">
-      <c r="A116" t="s" s="2">
-        <v>628</v>
-      </c>
-      <c r="B116" t="s" s="2">
-        <v>629</v>
-      </c>
-      <c r="C116" s="2"/>
-      <c r="D116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E116" s="2"/>
-      <c r="F116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K116" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L116" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="M116" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="N116" s="2"/>
-      <c r="O116" s="2"/>
-      <c r="P116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q116" s="2"/>
-      <c r="R116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB116" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="AC116" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="AD116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE116" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AF116" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG116" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH116" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ116" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO116" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP116" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="117" hidden="true">
-      <c r="A117" t="s" s="2">
-        <v>630</v>
-      </c>
-      <c r="B117" t="s" s="2">
-        <v>631</v>
-      </c>
-      <c r="C117" s="2"/>
-      <c r="D117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E117" s="2"/>
-      <c r="F117" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G117" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K117" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="L117" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="M117" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N117" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="O117" s="2"/>
-      <c r="P117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q117" s="2"/>
-      <c r="R117" t="s" s="2">
-        <v>632</v>
-      </c>
-      <c r="S117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF117" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="AG117" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AH117" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN117" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO117" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP117" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="118" hidden="true">
-      <c r="A118" t="s" s="2">
-        <v>633</v>
-      </c>
-      <c r="B118" t="s" s="2">
-        <v>634</v>
-      </c>
-      <c r="C118" s="2"/>
-      <c r="D118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E118" s="2"/>
-      <c r="F118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G118" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K118" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="L118" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="M118" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="N118" s="2"/>
-      <c r="O118" s="2"/>
-      <c r="P118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q118" s="2"/>
-      <c r="R118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S118" t="s" s="2">
-        <v>635</v>
-      </c>
-      <c r="T118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF118" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="AG118" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH118" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ118" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN118" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO118" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP118" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="119" hidden="true">
-      <c r="A119" t="s" s="2">
-        <v>636</v>
-      </c>
-      <c r="B119" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="C119" t="s" s="2">
-        <v>637</v>
-      </c>
-      <c r="D119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E119" s="2"/>
-      <c r="F119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G119" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K119" t="s" s="2">
-        <v>638</v>
-      </c>
-      <c r="L119" t="s" s="2">
-        <v>639</v>
-      </c>
-      <c r="M119" t="s" s="2">
-        <v>640</v>
-      </c>
-      <c r="N119" t="s" s="2">
-        <v>641</v>
-      </c>
-      <c r="O119" s="2"/>
-      <c r="P119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q119" s="2"/>
-      <c r="R119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF119" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG119" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH119" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI119" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="AJ119" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO119" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP119" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="120" hidden="true">
-      <c r="A120" t="s" s="2">
-        <v>642</v>
-      </c>
-      <c r="B120" t="s" s="2">
-        <v>627</v>
-      </c>
-      <c r="C120" s="2"/>
-      <c r="D120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E120" s="2"/>
-      <c r="F120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G120" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K120" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="L120" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="M120" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="N120" s="2"/>
-      <c r="O120" s="2"/>
-      <c r="P120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q120" s="2"/>
-      <c r="R120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF120" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="AG120" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH120" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN120" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="AO120" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP120" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="121" hidden="true">
-      <c r="A121" t="s" s="2">
-        <v>643</v>
-      </c>
-      <c r="B121" t="s" s="2">
-        <v>629</v>
-      </c>
-      <c r="C121" s="2"/>
-      <c r="D121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E121" s="2"/>
-      <c r="F121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K121" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L121" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="M121" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="N121" s="2"/>
-      <c r="O121" s="2"/>
-      <c r="P121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q121" s="2"/>
-      <c r="R121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB121" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="AC121" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="AD121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE121" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AF121" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG121" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH121" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ121" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO121" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP121" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="122" hidden="true">
-      <c r="A122" t="s" s="2">
-        <v>644</v>
-      </c>
-      <c r="B122" t="s" s="2">
-        <v>631</v>
-      </c>
-      <c r="C122" s="2"/>
-      <c r="D122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E122" s="2"/>
-      <c r="F122" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G122" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K122" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="L122" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="M122" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N122" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="O122" s="2"/>
-      <c r="P122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q122" s="2"/>
-      <c r="R122" t="s" s="2">
-        <v>645</v>
-      </c>
-      <c r="S122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF122" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="AG122" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AH122" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN122" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO122" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP122" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="s" s="2">
-        <v>646</v>
-      </c>
-      <c r="B123" t="s" s="2">
-        <v>634</v>
-      </c>
-      <c r="C123" s="2"/>
-      <c r="D123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E123" s="2"/>
-      <c r="F123" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G123" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H123" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K123" t="s" s="2">
-        <v>474</v>
-      </c>
-      <c r="L123" t="s" s="2">
-        <v>647</v>
-      </c>
-      <c r="M123" t="s" s="2">
-        <v>640</v>
-      </c>
-      <c r="N123" s="2"/>
-      <c r="O123" s="2"/>
-      <c r="P123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q123" s="2"/>
-      <c r="R123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF123" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="AG123" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH123" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ123" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN123" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO123" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP123" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="124" hidden="true">
-      <c r="A124" t="s" s="2">
-        <v>648</v>
-      </c>
-      <c r="B124" t="s" s="2">
-        <v>595</v>
-      </c>
-      <c r="C124" s="2"/>
-      <c r="D124" t="s" s="2">
-        <v>531</v>
-      </c>
-      <c r="E124" s="2"/>
-      <c r="F124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G124" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I124" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="J124" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K124" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L124" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="M124" t="s" s="2">
-        <v>533</v>
-      </c>
-      <c r="N124" t="s" s="2">
-        <v>227</v>
-      </c>
-      <c r="O124" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="P124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q124" s="2"/>
-      <c r="R124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF124" t="s" s="2">
-        <v>534</v>
-      </c>
-      <c r="AG124" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH124" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ124" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN124" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO124" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP124" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="s" s="2">
-        <v>649</v>
-      </c>
-      <c r="B125" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="C125" s="2"/>
-      <c r="D125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E125" s="2"/>
-      <c r="F125" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G125" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H125" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J125" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K125" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="L125" t="s" s="2">
-        <v>650</v>
-      </c>
-      <c r="M125" t="s" s="2">
-        <v>598</v>
-      </c>
-      <c r="N125" t="s" s="2">
-        <v>599</v>
-      </c>
-      <c r="O125" t="s" s="2">
-        <v>377</v>
-      </c>
-      <c r="P125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q125" s="2"/>
-      <c r="R125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X125" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="Y125" t="s" s="2">
-        <v>600</v>
-      </c>
-      <c r="Z125" t="s" s="2">
-        <v>601</v>
-      </c>
-      <c r="AA125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF125" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="AG125" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AH125" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ125" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK125" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL125" t="s" s="2">
-        <v>602</v>
-      </c>
-      <c r="AM125" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="AN125" t="s" s="2">
-        <v>383</v>
-      </c>
-      <c r="AO125" t="s" s="2">
-        <v>384</v>
-      </c>
-      <c r="AP125" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="s" s="2">
-        <v>651</v>
-      </c>
-      <c r="B126" t="s" s="2">
-        <v>603</v>
-      </c>
-      <c r="C126" s="2"/>
-      <c r="D126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E126" s="2"/>
-      <c r="F126" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G126" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H126" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J126" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K126" t="s" s="2">
-        <v>442</v>
-      </c>
-      <c r="L126" t="s" s="2">
-        <v>652</v>
-      </c>
-      <c r="M126" t="s" s="2">
-        <v>444</v>
-      </c>
-      <c r="N126" t="s" s="2">
-        <v>605</v>
-      </c>
-      <c r="O126" t="s" s="2">
-        <v>446</v>
-      </c>
-      <c r="P126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q126" s="2"/>
-      <c r="R126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF126" t="s" s="2">
-        <v>603</v>
-      </c>
-      <c r="AG126" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH126" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ126" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL126" t="s" s="2">
-        <v>606</v>
-      </c>
-      <c r="AM126" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="AN126" t="s" s="2">
-        <v>450</v>
-      </c>
-      <c r="AO126" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP126" t="s" s="2">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="127" hidden="true">
-      <c r="A127" t="s" s="2">
-        <v>653</v>
-      </c>
-      <c r="B127" t="s" s="2">
-        <v>607</v>
-      </c>
-      <c r="C127" s="2"/>
-      <c r="D127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E127" s="2"/>
-      <c r="F127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G127" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K127" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="L127" t="s" s="2">
-        <v>608</v>
-      </c>
-      <c r="M127" t="s" s="2">
-        <v>609</v>
-      </c>
-      <c r="N127" t="s" s="2">
-        <v>610</v>
-      </c>
-      <c r="O127" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="P127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q127" s="2"/>
-      <c r="R127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X127" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="Y127" t="s" s="2">
-        <v>457</v>
-      </c>
-      <c r="Z127" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="AA127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF127" t="s" s="2">
-        <v>607</v>
-      </c>
-      <c r="AG127" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH127" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI127" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="AJ127" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM127" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AN127" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="AO127" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP127" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="s" s="2">
-        <v>654</v>
-      </c>
-      <c r="B128" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="C128" s="2"/>
-      <c r="D128" t="s" s="2">
-        <v>462</v>
-      </c>
-      <c r="E128" s="2"/>
-      <c r="F128" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G128" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H128" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K128" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="L128" t="s" s="2">
-        <v>463</v>
-      </c>
-      <c r="M128" t="s" s="2">
-        <v>464</v>
-      </c>
-      <c r="N128" t="s" s="2">
-        <v>465</v>
-      </c>
-      <c r="O128" t="s" s="2">
-        <v>466</v>
-      </c>
-      <c r="P128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q128" s="2"/>
-      <c r="R128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X128" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="Y128" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="Z128" t="s" s="2">
-        <v>468</v>
-      </c>
-      <c r="AA128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF128" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="AG128" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH128" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ128" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL128" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="AM128" t="s" s="2">
-        <v>470</v>
-      </c>
-      <c r="AN128" t="s" s="2">
-        <v>471</v>
-      </c>
-      <c r="AO128" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP128" t="s" s="2">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="129" hidden="true">
-      <c r="A129" t="s" s="2">
-        <v>655</v>
-      </c>
-      <c r="B129" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="C129" s="2"/>
-      <c r="D129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E129" s="2"/>
-      <c r="F129" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G129" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K129" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="L129" t="s" s="2">
-        <v>614</v>
-      </c>
-      <c r="M129" t="s" s="2">
-        <v>615</v>
-      </c>
-      <c r="N129" t="s" s="2">
-        <v>523</v>
-      </c>
-      <c r="O129" t="s" s="2">
-        <v>524</v>
-      </c>
-      <c r="P129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q129" s="2"/>
-      <c r="R129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF129" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="AG129" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH129" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ129" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM129" t="s" s="2">
-        <v>526</v>
-      </c>
-      <c r="AN129" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="AO129" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP129" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="130" hidden="true">
-      <c r="A130" t="s" s="2">
-        <v>656</v>
-      </c>
-      <c r="B130" t="s" s="2">
-        <v>585</v>
-      </c>
-      <c r="C130" t="s" s="2">
-        <v>657</v>
-      </c>
-      <c r="D130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E130" s="2"/>
-      <c r="F130" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G130" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J130" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K130" t="s" s="2">
-        <v>520</v>
-      </c>
-      <c r="L130" t="s" s="2">
-        <v>658</v>
-      </c>
-      <c r="M130" t="s" s="2">
-        <v>587</v>
-      </c>
-      <c r="N130" t="s" s="2">
-        <v>588</v>
-      </c>
-      <c r="O130" t="s" s="2">
-        <v>589</v>
-      </c>
-      <c r="P130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q130" s="2"/>
-      <c r="R130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF130" t="s" s="2">
-        <v>585</v>
-      </c>
-      <c r="AG130" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH130" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ130" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM130" t="s" s="2">
-        <v>591</v>
-      </c>
-      <c r="AN130" t="s" s="2">
-        <v>592</v>
-      </c>
-      <c r="AO130" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP130" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="131" hidden="true">
-      <c r="A131" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="B131" t="s" s="2">
-        <v>593</v>
-      </c>
-      <c r="C131" s="2"/>
-      <c r="D131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E131" s="2"/>
-      <c r="F131" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G131" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K131" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="L131" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="M131" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="N131" s="2"/>
-      <c r="O131" s="2"/>
-      <c r="P131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q131" s="2"/>
-      <c r="R131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF131" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="AG131" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH131" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN131" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="AO131" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP131" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="132" hidden="true">
-      <c r="A132" t="s" s="2">
-        <v>660</v>
-      </c>
-      <c r="B132" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="C132" s="2"/>
-      <c r="D132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E132" s="2"/>
-      <c r="F132" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G132" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K132" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L132" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="M132" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="N132" s="2"/>
-      <c r="O132" s="2"/>
-      <c r="P132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q132" s="2"/>
-      <c r="R132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB132" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="AC132" s="2"/>
-      <c r="AD132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE132" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AF132" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG132" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH132" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ132" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO132" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP132" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="133" hidden="true">
-      <c r="A133" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="B133" t="s" s="2">
-        <v>594</v>
-      </c>
-      <c r="C133" t="s" s="2">
-        <v>622</v>
-      </c>
-      <c r="D133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E133" s="2"/>
-      <c r="F133" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G133" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K133" t="s" s="2">
-        <v>623</v>
-      </c>
-      <c r="L133" t="s" s="2">
-        <v>624</v>
-      </c>
-      <c r="M133" t="s" s="2">
-        <v>625</v>
-      </c>
-      <c r="N133" s="2"/>
-      <c r="O133" s="2"/>
-      <c r="P133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q133" s="2"/>
-      <c r="R133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF133" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG133" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH133" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI133" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="AJ133" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO133" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP133" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="134" hidden="true">
-      <c r="A134" t="s" s="2">
-        <v>662</v>
-      </c>
-      <c r="B134" t="s" s="2">
-        <v>627</v>
-      </c>
-      <c r="C134" s="2"/>
-      <c r="D134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E134" s="2"/>
-      <c r="F134" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G134" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K134" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="L134" t="s" s="2">
-        <v>154</v>
-      </c>
-      <c r="M134" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="N134" s="2"/>
-      <c r="O134" s="2"/>
-      <c r="P134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q134" s="2"/>
-      <c r="R134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF134" t="s" s="2">
-        <v>156</v>
-      </c>
-      <c r="AG134" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH134" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN134" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="AO134" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP134" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="135" hidden="true">
-      <c r="A135" t="s" s="2">
-        <v>663</v>
-      </c>
-      <c r="B135" t="s" s="2">
-        <v>629</v>
-      </c>
-      <c r="C135" s="2"/>
-      <c r="D135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E135" s="2"/>
-      <c r="F135" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G135" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K135" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L135" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="M135" t="s" s="2">
-        <v>140</v>
-      </c>
-      <c r="N135" s="2"/>
-      <c r="O135" s="2"/>
-      <c r="P135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q135" s="2"/>
-      <c r="R135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB135" t="s" s="2">
-        <v>141</v>
-      </c>
-      <c r="AC135" t="s" s="2">
-        <v>161</v>
-      </c>
-      <c r="AD135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE135" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="AF135" t="s" s="2">
-        <v>162</v>
-      </c>
-      <c r="AG135" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH135" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ135" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AO135" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP135" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="136" hidden="true">
-      <c r="A136" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="B136" t="s" s="2">
-        <v>631</v>
-      </c>
-      <c r="C136" s="2"/>
-      <c r="D136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E136" s="2"/>
-      <c r="F136" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G136" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K136" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="L136" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="M136" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N136" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="O136" s="2"/>
-      <c r="P136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q136" s="2"/>
-      <c r="R136" t="s" s="2">
-        <v>632</v>
-      </c>
-      <c r="S136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF136" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="AG136" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AH136" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN136" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO136" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP136" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="137" hidden="true">
-      <c r="A137" t="s" s="2">
-        <v>665</v>
-      </c>
-      <c r="B137" t="s" s="2">
-        <v>634</v>
-      </c>
-      <c r="C137" s="2"/>
-      <c r="D137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E137" s="2"/>
-      <c r="F137" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G137" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K137" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="L137" t="s" s="2">
-        <v>177</v>
-      </c>
-      <c r="M137" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="N137" s="2"/>
-      <c r="O137" s="2"/>
-      <c r="P137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q137" s="2"/>
-      <c r="R137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S137" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="T137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF137" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="AG137" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH137" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ137" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN137" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO137" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP137" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="138" hidden="true">
-      <c r="A138" t="s" s="2">
-        <v>667</v>
-      </c>
-      <c r="B138" t="s" s="2">
-        <v>595</v>
-      </c>
-      <c r="C138" s="2"/>
-      <c r="D138" t="s" s="2">
-        <v>531</v>
-      </c>
-      <c r="E138" s="2"/>
-      <c r="F138" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G138" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I138" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="J138" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K138" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="L138" t="s" s="2">
-        <v>532</v>
-      </c>
-      <c r="M138" t="s" s="2">
-        <v>533</v>
-      </c>
-      <c r="N138" t="s" s="2">
-        <v>227</v>
-      </c>
-      <c r="O138" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="P138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q138" s="2"/>
-      <c r="R138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF138" t="s" s="2">
-        <v>534</v>
-      </c>
-      <c r="AG138" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH138" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ138" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="AK138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AN138" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AO138" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP138" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="s" s="2">
-        <v>668</v>
-      </c>
-      <c r="B139" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="C139" s="2"/>
-      <c r="D139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E139" s="2"/>
-      <c r="F139" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G139" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H139" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J139" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K139" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="L139" t="s" s="2">
-        <v>650</v>
-      </c>
-      <c r="M139" t="s" s="2">
-        <v>598</v>
-      </c>
-      <c r="N139" t="s" s="2">
-        <v>599</v>
-      </c>
-      <c r="O139" t="s" s="2">
-        <v>377</v>
-      </c>
-      <c r="P139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q139" s="2"/>
-      <c r="R139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X139" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="Y139" t="s" s="2">
-        <v>600</v>
-      </c>
-      <c r="Z139" t="s" s="2">
-        <v>601</v>
-      </c>
-      <c r="AA139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF139" t="s" s="2">
-        <v>596</v>
-      </c>
-      <c r="AG139" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AH139" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ139" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK139" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL139" t="s" s="2">
-        <v>602</v>
-      </c>
-      <c r="AM139" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="AN139" t="s" s="2">
-        <v>383</v>
-      </c>
-      <c r="AO139" t="s" s="2">
-        <v>384</v>
-      </c>
-      <c r="AP139" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="s" s="2">
-        <v>669</v>
-      </c>
-      <c r="B140" t="s" s="2">
-        <v>603</v>
-      </c>
-      <c r="C140" s="2"/>
-      <c r="D140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E140" s="2"/>
-      <c r="F140" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="G140" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H140" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J140" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="K140" t="s" s="2">
-        <v>442</v>
-      </c>
-      <c r="L140" t="s" s="2">
-        <v>652</v>
-      </c>
-      <c r="M140" t="s" s="2">
-        <v>444</v>
-      </c>
-      <c r="N140" t="s" s="2">
-        <v>605</v>
-      </c>
-      <c r="O140" t="s" s="2">
-        <v>446</v>
-      </c>
-      <c r="P140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q140" s="2"/>
-      <c r="R140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF140" t="s" s="2">
-        <v>603</v>
-      </c>
-      <c r="AG140" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH140" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ140" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL140" t="s" s="2">
-        <v>606</v>
-      </c>
-      <c r="AM140" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="AN140" t="s" s="2">
-        <v>450</v>
-      </c>
-      <c r="AO140" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP140" t="s" s="2">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="141" hidden="true">
-      <c r="A141" t="s" s="2">
-        <v>670</v>
-      </c>
-      <c r="B141" t="s" s="2">
-        <v>607</v>
-      </c>
-      <c r="C141" s="2"/>
-      <c r="D141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E141" s="2"/>
-      <c r="F141" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G141" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K141" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="L141" t="s" s="2">
-        <v>608</v>
-      </c>
-      <c r="M141" t="s" s="2">
-        <v>609</v>
-      </c>
-      <c r="N141" t="s" s="2">
-        <v>610</v>
-      </c>
-      <c r="O141" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="P141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q141" s="2"/>
-      <c r="R141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X141" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="Y141" t="s" s="2">
-        <v>457</v>
-      </c>
-      <c r="Z141" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="AA141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF141" t="s" s="2">
-        <v>607</v>
-      </c>
-      <c r="AG141" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH141" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AI141" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="AJ141" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM141" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AN141" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="AO141" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP141" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="s" s="2">
-        <v>671</v>
-      </c>
-      <c r="B142" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="C142" s="2"/>
-      <c r="D142" t="s" s="2">
-        <v>462</v>
-      </c>
-      <c r="E142" s="2"/>
-      <c r="F142" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G142" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="H142" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="I142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K142" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="L142" t="s" s="2">
-        <v>463</v>
-      </c>
-      <c r="M142" t="s" s="2">
-        <v>464</v>
-      </c>
-      <c r="N142" t="s" s="2">
-        <v>465</v>
-      </c>
-      <c r="O142" t="s" s="2">
-        <v>466</v>
-      </c>
-      <c r="P142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q142" s="2"/>
-      <c r="R142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X142" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="Y142" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="Z142" t="s" s="2">
-        <v>468</v>
-      </c>
-      <c r="AA142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF142" t="s" s="2">
-        <v>611</v>
-      </c>
-      <c r="AG142" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH142" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ142" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL142" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="AM142" t="s" s="2">
-        <v>470</v>
-      </c>
-      <c r="AN142" t="s" s="2">
-        <v>471</v>
-      </c>
-      <c r="AO142" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP142" t="s" s="2">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="143" hidden="true">
-      <c r="A143" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="B143" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="C143" s="2"/>
-      <c r="D143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="E143" s="2"/>
-      <c r="F143" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G143" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="I143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="J143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K143" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="L143" t="s" s="2">
-        <v>614</v>
-      </c>
-      <c r="M143" t="s" s="2">
-        <v>615</v>
-      </c>
-      <c r="N143" t="s" s="2">
-        <v>523</v>
-      </c>
-      <c r="O143" t="s" s="2">
-        <v>524</v>
-      </c>
-      <c r="P143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Q143" s="2"/>
-      <c r="R143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="S143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="T143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="U143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="V143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="W143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="X143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Y143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="Z143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AA143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AB143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AC143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AD143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AE143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AF143" t="s" s="2">
-        <v>613</v>
-      </c>
-      <c r="AG143" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH143" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AJ143" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AL143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AM143" t="s" s="2">
-        <v>526</v>
-      </c>
-      <c r="AN143" t="s" s="2">
-        <v>527</v>
-      </c>
-      <c r="AO143" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AP143" t="s" s="2">
-        <v>82</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AP143">
+  <autoFilter ref="A1:AP110">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -19629,7 +15490,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI142">
+  <conditionalFormatting sqref="A2:AI109">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>